<commit_message>
data: sync PC-server-0148 2026-09-24 17:48
</commit_message>
<xml_diff>
--- a/data/美团.xlsx
+++ b/data/美团.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2661,179 +2661,165 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
+      <c r="A94" t="n">
+        <v>934</v>
       </c>
       <c r="B94" s="1" t="n">
-        <v>46282.45922453704</v>
+        <v>46286.48706018519</v>
       </c>
       <c r="C94" s="1" t="n">
-        <v>46282.46618055556</v>
+        <v>46286.49402777778</v>
       </c>
       <c r="D94" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率23，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>934</v>
+      </c>
+      <c r="B95" s="1" t="n">
+        <v>46286.50042824074</v>
+      </c>
+      <c r="C95" s="1" t="n">
+        <v>46286.50737268518</v>
+      </c>
+      <c r="D95" t="n">
+        <v>10</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率31，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>934</v>
+      </c>
+      <c r="B96" s="1" t="n">
+        <v>46286.5983912037</v>
+      </c>
+      <c r="C96" s="1" t="n">
+        <v>46286.60533564815</v>
+      </c>
+      <c r="D96" t="n">
+        <v>10</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率16，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>934</v>
+      </c>
+      <c r="B97" s="1" t="n">
+        <v>46287.11172453704</v>
+      </c>
+      <c r="C97" s="1" t="n">
+        <v>46287.11868055556</v>
+      </c>
+      <c r="D97" t="n">
         <v>10.02</v>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>【美团】站点934：预定验价变价率18，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B95" s="1" t="n">
-        <v>46282.473125</v>
-      </c>
-      <c r="C95" s="1" t="n">
-        <v>46282.4799537037</v>
-      </c>
-      <c r="D95" t="n">
-        <v>9.83</v>
-      </c>
-      <c r="E95" t="inlineStr">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率26，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>934</v>
+      </c>
+      <c r="B98" s="1" t="n">
+        <v>46287.12581018519</v>
+      </c>
+      <c r="C98" s="1" t="n">
+        <v>46287.13274305555</v>
+      </c>
+      <c r="D98" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率28，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>934</v>
+      </c>
+      <c r="B99" s="1" t="n">
+        <v>46287.30594907407</v>
+      </c>
+      <c r="C99" s="1" t="n">
+        <v>46287.31291666667</v>
+      </c>
+      <c r="D99" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>【美团】站点934：预定验价变价率17，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B96" s="1" t="n">
-        <v>46282.97300925926</v>
-      </c>
-      <c r="C96" s="1" t="n">
-        <v>46282.97993055556</v>
-      </c>
-      <c r="D96" t="n">
-        <v>9.970000000000001</v>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>【美团】站点934：预定验价变价率18，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B97" s="1" t="n">
-        <v>46286.48706018519</v>
-      </c>
-      <c r="C97" s="1" t="n">
-        <v>46286.49402777778</v>
-      </c>
-      <c r="D97" t="n">
-        <v>10.03</v>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>【美团】站点934：预定验价变价率23，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B98" s="1" t="n">
-        <v>46286.50042824074</v>
-      </c>
-      <c r="C98" s="1" t="n">
-        <v>46286.50737268518</v>
-      </c>
-      <c r="D98" t="n">
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>934</v>
+      </c>
+      <c r="B100" s="1" t="n">
+        <v>46287.32052083333</v>
+      </c>
+      <c r="C100" s="1" t="n">
+        <v>46287.32746527778</v>
+      </c>
+      <c r="D100" t="n">
         <v>10</v>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>【美团】站点934：预定验价变价率31，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B99" s="1" t="n">
-        <v>46286.5983912037</v>
-      </c>
-      <c r="C99" s="1" t="n">
-        <v>46286.60533564815</v>
-      </c>
-      <c r="D99" t="n">
-        <v>10</v>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>【美团】站点934：预定验价变价率16，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>【美团】站点934恢复上线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>934</t>
-        </is>
-      </c>
-      <c r="B100" s="1" t="n">
-        <v>46287.11172453704</v>
-      </c>
-      <c r="C100" s="1" t="n">
-        <v>46287.11868055556</v>
-      </c>
-      <c r="D100" t="n">
-        <v>10.02</v>
-      </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>【美团】站点934：预定验价变价率26，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+          <t>【美团】站点934：预定验价变价率20，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -2849,17 +2835,17 @@
         </is>
       </c>
       <c r="B101" s="1" t="n">
-        <v>46287.12581018519</v>
+        <v>46282.97300925926</v>
       </c>
       <c r="C101" s="1" t="n">
-        <v>46287.13274305555</v>
+        <v>46282.97993055556</v>
       </c>
       <c r="D101" t="n">
-        <v>9.98</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>【美团】站点934：预定验价变价率28，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+          <t>【美团】站点934：预定验价变价率18，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -2875,17 +2861,17 @@
         </is>
       </c>
       <c r="B102" s="1" t="n">
-        <v>46287.30594907407</v>
+        <v>46286.48706018519</v>
       </c>
       <c r="C102" s="1" t="n">
-        <v>46287.31291666667</v>
+        <v>46286.49402777778</v>
       </c>
       <c r="D102" t="n">
         <v>10.03</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>【美团】站点934：预定验价变价率17，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+          <t>【美团】站点934：预定验价变价率23，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -2901,20 +2887,332 @@
         </is>
       </c>
       <c r="B103" s="1" t="n">
-        <v>46287.32052083333</v>
+        <v>46286.50042824074</v>
       </c>
       <c r="C103" s="1" t="n">
-        <v>46287.32746527778</v>
+        <v>46286.50737268518</v>
       </c>
       <c r="D103" t="n">
         <v>10</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
+          <t>【美团】站点934：预定验价变价率31，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="n">
+        <v>46286.5983912037</v>
+      </c>
+      <c r="C104" s="1" t="n">
+        <v>46286.60533564815</v>
+      </c>
+      <c r="D104" t="n">
+        <v>10</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率16，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="n">
+        <v>46287.11172453704</v>
+      </c>
+      <c r="C105" s="1" t="n">
+        <v>46287.11868055556</v>
+      </c>
+      <c r="D105" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率26，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="n">
+        <v>46287.12581018519</v>
+      </c>
+      <c r="C106" s="1" t="n">
+        <v>46287.13274305555</v>
+      </c>
+      <c r="D106" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率28，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="n">
+        <v>46287.30594907407</v>
+      </c>
+      <c r="C107" s="1" t="n">
+        <v>46287.31291666667</v>
+      </c>
+      <c r="D107" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率17，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="n">
+        <v>46287.32052083333</v>
+      </c>
+      <c r="C108" s="1" t="n">
+        <v>46287.32746527778</v>
+      </c>
+      <c r="D108" t="n">
+        <v>10</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
           <t>【美团】站点934：预定验价变价率20，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="n">
+        <v>46287.38972222222</v>
+      </c>
+      <c r="C109" s="1" t="n">
+        <v>46287.39673611111</v>
+      </c>
+      <c r="D109" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率27，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="n">
+        <v>46287.40336805556</v>
+      </c>
+      <c r="C110" s="1" t="n">
+        <v>46287.41027777778</v>
+      </c>
+      <c r="D110" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率20，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="n">
+        <v>46287.41793981481</v>
+      </c>
+      <c r="C111" s="1" t="n">
+        <v>46287.42490740741</v>
+      </c>
+      <c r="D111" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率21，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="n">
+        <v>46289.11177083333</v>
+      </c>
+      <c r="C112" s="1" t="n">
+        <v>46289.11864583333</v>
+      </c>
+      <c r="D112" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率18，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="n">
+        <v>46289.1255787037</v>
+      </c>
+      <c r="C113" s="1" t="n">
+        <v>46289.1325</v>
+      </c>
+      <c r="D113" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率21，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="n">
+        <v>46289.29210648148</v>
+      </c>
+      <c r="C114" s="1" t="n">
+        <v>46289.2990625</v>
+      </c>
+      <c r="D114" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率16，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>【美团】站点934恢复上线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>934</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="n">
+        <v>46289.30592592592</v>
+      </c>
+      <c r="C115" s="1" t="n">
+        <v>46289.31285879629</v>
+      </c>
+      <c r="D115" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>【美团】站点934：预定验价变价率20，下线，请及时处理。具体原因及日志请查看「美团机票商家端系统-合作商监控-预定记录」</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
         <is>
           <t>【美团】站点934恢复上线。</t>
         </is>

</xml_diff>